<commit_message>
Move CLI config to ~/.config/htbm/cli and use English sheet headers.
Centralize config paths under htbm, regenerate spreadsheet templates in English, update docs/worklog, and refresh README dashboard branding assets.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/examples/sheets/htb_machines_example.xlsx
+++ b/examples/sheets/htb_machines_example.xlsx
@@ -27,31 +27,31 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="261">
   <si>
-    <t>Nombre</t>
-  </si>
-  <si>
-    <t>Titulo</t>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Title</t>
   </si>
   <si>
     <t>OS</t>
   </si>
   <si>
-    <t>Dificultad</t>
-  </si>
-  <si>
-    <t>Tecnicas</t>
-  </si>
-  <si>
-    <t>Fecha</t>
-  </si>
-  <si>
-    <t>Activa</t>
+    <t>Difficulty</t>
+  </si>
+  <si>
+    <t>Techniques</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Active</t>
   </si>
   <si>
     <t>URL</t>
   </si>
   <si>
-    <t>Hecha</t>
+    <t>Done</t>
   </si>
   <si>
     <t>airtouch</t>

</xml_diff>